<commit_message>
Modified code for JTS and Final code for France
</commit_message>
<xml_diff>
--- a/Data/Template for Complted Country/testDataHungry.xlsx
+++ b/Data/Template for Complted Country/testDataHungry.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{59C643C9-9EC0-4514-AB9A-37245B438818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABED2A57-5752-4DE4-B1E9-E1551B997916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,7 +11,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1680,7 +1679,7 @@
       </c>
       <c r="K2" s="19">
         <f t="shared" ref="K2:K15" ca="1" si="0">TODAY()-31</f>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L2" s="20" t="s">
         <v>96</v>
@@ -1723,7 +1722,7 @@
       </c>
       <c r="Y2" s="19">
         <f t="shared" ref="Y2:Y15" ca="1" si="1">K2</f>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z2" s="18" t="s">
         <v>109</v>
@@ -1757,11 +1756,11 @@
       </c>
       <c r="AJ2" s="31">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AK2" s="31">
         <f t="shared" ref="AK2:AK15" ca="1" si="2">Y2+90</f>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL2" s="18" t="s">
         <v>116</v>
@@ -1799,15 +1798,15 @@
       </c>
       <c r="AW2" s="33">
         <f t="shared" ref="AW2:AW15" ca="1" si="4">Y2-1</f>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX2" s="33">
         <f t="shared" ref="AX2:AX15" ca="1" si="5">Y2-1</f>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY2" s="34">
         <f t="shared" ref="AY2:AY7" ca="1" si="6">AJ2</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AZ2" s="24" t="s">
         <v>96</v>
@@ -1977,7 +1976,7 @@
       </c>
       <c r="K3" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L3" s="20" t="s">
         <v>96</v>
@@ -2020,7 +2019,7 @@
       </c>
       <c r="Y3" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z3" s="18" t="s">
         <v>109</v>
@@ -2057,7 +2056,7 @@
       </c>
       <c r="AK3" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL3" s="18" t="s">
         <v>116</v>
@@ -2095,11 +2094,11 @@
       </c>
       <c r="AW3" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX3" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY3" s="34" t="str">
         <f t="shared" si="6"/>
@@ -2239,7 +2238,7 @@
       </c>
       <c r="CR3" s="48">
         <f ca="1">TODAY()-1500</f>
-        <v>44240</v>
+        <v>44254</v>
       </c>
       <c r="CS3" s="30" t="s">
         <v>162</v>
@@ -2275,7 +2274,7 @@
       </c>
       <c r="K4" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L4" s="20" t="s">
         <v>96</v>
@@ -2318,7 +2317,7 @@
       </c>
       <c r="Y4" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z4" s="18" t="s">
         <v>109</v>
@@ -2355,7 +2354,7 @@
       </c>
       <c r="AK4" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL4" s="18" t="s">
         <v>116</v>
@@ -2393,11 +2392,11 @@
       </c>
       <c r="AW4" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX4" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY4" s="50" t="str">
         <f t="shared" si="6"/>
@@ -2572,7 +2571,7 @@
       </c>
       <c r="K5" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L5" s="20" t="s">
         <v>96</v>
@@ -2615,7 +2614,7 @@
       </c>
       <c r="Y5" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z5" s="18" t="s">
         <v>109</v>
@@ -2649,11 +2648,11 @@
       </c>
       <c r="AJ5" s="31">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AK5" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL5" s="18" t="s">
         <v>116</v>
@@ -2691,15 +2690,15 @@
       </c>
       <c r="AW5" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX5" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY5" s="34">
         <f t="shared" ca="1" si="6"/>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AZ5" s="24" t="s">
         <v>96</v>
@@ -2869,7 +2868,7 @@
       </c>
       <c r="K6" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L6" s="20" t="s">
         <v>96</v>
@@ -2912,7 +2911,7 @@
       </c>
       <c r="Y6" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z6" s="18" t="s">
         <v>109</v>
@@ -2949,7 +2948,7 @@
       </c>
       <c r="AK6" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL6" s="18" t="s">
         <v>116</v>
@@ -2987,11 +2986,11 @@
       </c>
       <c r="AW6" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX6" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY6" s="34" t="str">
         <f t="shared" si="6"/>
@@ -3165,7 +3164,7 @@
       </c>
       <c r="K7" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L7" s="20" t="s">
         <v>96</v>
@@ -3208,7 +3207,7 @@
       </c>
       <c r="Y7" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z7" s="18" t="s">
         <v>109</v>
@@ -3242,11 +3241,11 @@
       </c>
       <c r="AJ7" s="31">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AK7" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL7" s="18" t="s">
         <v>116</v>
@@ -3284,15 +3283,15 @@
       </c>
       <c r="AW7" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX7" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY7" s="34">
         <f t="shared" ca="1" si="6"/>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AZ7" s="24" t="s">
         <v>96</v>
@@ -3462,7 +3461,7 @@
       </c>
       <c r="K8" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L8" s="20" t="s">
         <v>96</v>
@@ -3505,7 +3504,7 @@
       </c>
       <c r="Y8" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z8" s="18" t="s">
         <v>109</v>
@@ -3542,7 +3541,7 @@
       </c>
       <c r="AK8" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL8" s="18" t="s">
         <v>116</v>
@@ -3580,11 +3579,11 @@
       </c>
       <c r="AW8" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX8" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY8" s="34" t="s">
         <v>110</v>
@@ -3723,7 +3722,7 @@
       </c>
       <c r="CR8" s="48">
         <f ca="1">TODAY()-1500</f>
-        <v>44240</v>
+        <v>44254</v>
       </c>
       <c r="CS8" s="30" t="s">
         <v>162</v>
@@ -3758,7 +3757,7 @@
       </c>
       <c r="K9" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L9" s="20" t="s">
         <v>96</v>
@@ -3801,7 +3800,7 @@
       </c>
       <c r="Y9" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z9" s="18" t="s">
         <v>109</v>
@@ -3835,11 +3834,11 @@
       </c>
       <c r="AJ9" s="31">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AK9" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL9" s="18" t="s">
         <v>116</v>
@@ -3877,15 +3876,15 @@
       </c>
       <c r="AW9" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX9" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY9" s="34">
         <f ca="1">AJ9</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AZ9" s="24" t="s">
         <v>96</v>
@@ -4055,7 +4054,7 @@
       </c>
       <c r="K10" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L10" s="20" t="s">
         <v>96</v>
@@ -4098,7 +4097,7 @@
       </c>
       <c r="Y10" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z10" s="18" t="s">
         <v>109</v>
@@ -4135,7 +4134,7 @@
       </c>
       <c r="AK10" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL10" s="18" t="s">
         <v>116</v>
@@ -4173,11 +4172,11 @@
       </c>
       <c r="AW10" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX10" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY10" s="34" t="s">
         <v>110</v>
@@ -4350,7 +4349,7 @@
       </c>
       <c r="K11" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L11" s="20" t="s">
         <v>96</v>
@@ -4393,7 +4392,7 @@
       </c>
       <c r="Y11" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z11" s="18" t="s">
         <v>109</v>
@@ -4427,11 +4426,11 @@
       </c>
       <c r="AJ11" s="31">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AK11" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL11" s="18" t="s">
         <v>116</v>
@@ -4469,15 +4468,15 @@
       </c>
       <c r="AW11" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX11" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY11" s="34">
         <f ca="1">AJ11</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AZ11" s="24" t="s">
         <v>96</v>
@@ -4613,7 +4612,7 @@
       </c>
       <c r="CR11" s="48">
         <f ca="1">TODAY()-1500</f>
-        <v>44240</v>
+        <v>44254</v>
       </c>
       <c r="CS11" s="30" t="s">
         <v>162</v>
@@ -4648,7 +4647,7 @@
       </c>
       <c r="K12" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L12" s="20" t="s">
         <v>96</v>
@@ -4691,7 +4690,7 @@
       </c>
       <c r="Y12" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z12" s="18" t="s">
         <v>109</v>
@@ -4728,7 +4727,7 @@
       </c>
       <c r="AK12" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL12" s="18" t="s">
         <v>116</v>
@@ -4766,11 +4765,11 @@
       </c>
       <c r="AW12" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX12" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY12" s="34" t="str">
         <f>AJ12</f>
@@ -4944,7 +4943,7 @@
       </c>
       <c r="K13" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L13" s="20" t="s">
         <v>96</v>
@@ -4987,7 +4986,7 @@
       </c>
       <c r="Y13" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z13" s="18" t="s">
         <v>109</v>
@@ -5021,11 +5020,11 @@
       </c>
       <c r="AJ13" s="31">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AK13" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL13" s="18" t="s">
         <v>116</v>
@@ -5063,15 +5062,15 @@
       </c>
       <c r="AW13" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX13" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY13" s="34">
         <f ca="1">AJ13</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AZ13" s="24" t="s">
         <v>96</v>
@@ -5241,7 +5240,7 @@
       </c>
       <c r="K14" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L14" s="20" t="s">
         <v>96</v>
@@ -5284,7 +5283,7 @@
       </c>
       <c r="Y14" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z14" s="18" t="s">
         <v>109</v>
@@ -5321,7 +5320,7 @@
       </c>
       <c r="AK14" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL14" s="18" t="s">
         <v>116</v>
@@ -5359,11 +5358,11 @@
       </c>
       <c r="AW14" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX14" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY14" s="34" t="str">
         <f>AJ14</f>
@@ -5537,7 +5536,7 @@
       </c>
       <c r="K15" s="19">
         <f t="shared" ca="1" si="0"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="L15" s="20" t="s">
         <v>96</v>
@@ -5580,7 +5579,7 @@
       </c>
       <c r="Y15" s="19">
         <f t="shared" ca="1" si="1"/>
-        <v>45709</v>
+        <v>45723</v>
       </c>
       <c r="Z15" s="18" t="s">
         <v>109</v>
@@ -5614,11 +5613,11 @@
       </c>
       <c r="AJ15" s="31">
         <f ca="1">TODAY()+365</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AK15" s="31">
         <f t="shared" ca="1" si="2"/>
-        <v>45799</v>
+        <v>45813</v>
       </c>
       <c r="AL15" s="18" t="s">
         <v>116</v>
@@ -5656,15 +5655,15 @@
       </c>
       <c r="AW15" s="33">
         <f t="shared" ca="1" si="4"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AX15" s="33">
         <f t="shared" ca="1" si="5"/>
-        <v>45708</v>
+        <v>45722</v>
       </c>
       <c r="AY15" s="34">
         <f ca="1">AJ15</f>
-        <v>46105</v>
+        <v>46119</v>
       </c>
       <c r="AZ15" s="24" t="s">
         <v>96</v>
@@ -5814,7 +5813,7 @@
     <row r="16" spans="1:100" ht="14.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AJ16" s="55"/>
     </row>
-    <row r="17" spans="36:36" ht="14.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="36:36" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AJ17" s="55"/>
     </row>
   </sheetData>

</xml_diff>